<commit_message>
feat: Cap nhat cot MA_LOAI mac dinh la TT cho toan bo danh muc thuoc gen file import
</commit_message>
<xml_diff>
--- a/CauHinh_NghiepVu_HMIS.xlsx
+++ b/CauHinh_NghiepVu_HMIS.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="yyyymmdd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -590,10 +591,10 @@
         <v>link</v>
       </c>
       <c r="F6" t="str">
-        <v>https://test-emr.vncare.vn</v>
+        <v>https://emr.vncare.vn/</v>
       </c>
       <c r="G6" t="str">
-        <v>https://test-emr.vncare.vn</v>
+        <v>https://emr.vncare.vn/</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -602,7 +603,7 @@
         <v>Bật</v>
       </c>
       <c r="J6" t="str">
-        <v>08/09/2026 11:08:36</v>
+        <v>14/10/2026 14:26:55</v>
       </c>
     </row>
     <row r="7">
@@ -622,10 +623,10 @@
         <v>username</v>
       </c>
       <c r="F7" t="str">
-        <v>84142.admin</v>
+        <v>11010.admin</v>
       </c>
       <c r="G7" t="str">
-        <v>84142.admin</v>
+        <v>11010.admin</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -634,7 +635,7 @@
         <v>Bật</v>
       </c>
       <c r="J7" t="str">
-        <v>08/09/2026 11:08:36</v>
+        <v>14/10/2026 14:26:55</v>
       </c>
     </row>
     <row r="8">
@@ -654,10 +655,10 @@
         <v>password</v>
       </c>
       <c r="F8" t="str">
-        <v>d7685c362a5646A*!</v>
+        <v>Emr@11010</v>
       </c>
       <c r="G8" t="str">
-        <v>d7685c362a5646A*!</v>
+        <v>Emr@11010</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -666,7 +667,7 @@
         <v>Bật</v>
       </c>
       <c r="J8" t="str">
-        <v>08/09/2026 11:08:36</v>
+        <v>14/10/2026 14:26:55</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -18483,7 +18484,7 @@
         <v>Bật</v>
       </c>
       <c r="J538" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="539" xml:space="preserve">
@@ -18516,7 +18517,7 @@
         <v>Bật</v>
       </c>
       <c r="J539" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="540" xml:space="preserve">
@@ -18550,7 +18551,7 @@
         <v>Bật</v>
       </c>
       <c r="J540" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="541" xml:space="preserve">
@@ -18584,7 +18585,7 @@
         <v>Bật</v>
       </c>
       <c r="J541" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="542" xml:space="preserve">
@@ -18618,7 +18619,7 @@
         <v>Bật</v>
       </c>
       <c r="J542" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="543" xml:space="preserve">
@@ -18638,7 +18639,7 @@
         <v>moDTNGT</v>
       </c>
       <c r="F543" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G543" t="str">
         <v>0</v>
@@ -18653,7 +18654,7 @@
         <v>Bật</v>
       </c>
       <c r="J543" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="544">
@@ -18685,7 +18686,7 @@
         <v>Bật</v>
       </c>
       <c r="J544" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="545" xml:space="preserve">
@@ -18718,7 +18719,7 @@
         <v>Bật</v>
       </c>
       <c r="J545" t="str">
-        <v>29/06/2026 11:23:19</v>
+        <v>11/10/2026 20:48:52</v>
       </c>
     </row>
     <row r="546" xml:space="preserve">

</xml_diff>

<commit_message>
feat: Them chuc nang Thiet lap Phieu in Bao cao dong bo hang loat cho cac tram y te da tich tren cong HMIS
</commit_message>
<xml_diff>
--- a/CauHinh_NghiepVu_HMIS.xlsx
+++ b/CauHinh_NghiepVu_HMIS.xlsx
@@ -32,9 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="yyyymmdd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -1694,7 +1693,7 @@
         <v>Bật</v>
       </c>
       <c r="J40" t="str">
-        <v>15/09/2026 22:56:24</v>
+        <v>15/10/2026 12:03:39</v>
       </c>
     </row>
     <row r="41">
@@ -1726,7 +1725,7 @@
         <v>Bật</v>
       </c>
       <c r="J41" t="str">
-        <v>15/09/2026 22:56:24</v>
+        <v>15/10/2026 12:03:39</v>
       </c>
     </row>
     <row r="42">
@@ -1758,7 +1757,7 @@
         <v>Bật</v>
       </c>
       <c r="J42" t="str">
-        <v>15/09/2026 22:56:24</v>
+        <v>15/10/2026 12:03:39</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -1785,14 +1784,15 @@
       </c>
       <c r="H43" t="str" xml:space="preserve">
         <v xml:space="preserve">Cấu hình cho phép tự động điền chiều cao, cân nặng… vv từ khám Lâm sàng vào mục khám Thể Lực
-            0: Cho phép tự động (mặc định)
-            1: Không cho phép tự động.</v>
+            0: Cho phép tự động (Chỉ tự động phân loại theo chiều cao cân nặng)
+            1: Không cho phép tự động.
+            2: Cho phép tự động (tự động phân loại theo chiều cao, cân nặng, huyết áp và mạch)</v>
       </c>
       <c r="I43" t="str">
         <v>Bật</v>
       </c>
       <c r="J43" t="str">
-        <v>15/09/2026 22:56:24</v>
+        <v>15/10/2026 12:03:39</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">

</xml_diff>